<commit_message>
n8n board refresh 2026-09-13T17:41:28Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-11 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-13 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.867</v>
+        <v>0.866</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>323.45</v>
+        <v>322.14</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>181.3001</v>
+        <v>183.9</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.784</v>
+        <v>0.752</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.78</v>
+        <v>0.775</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04947000026702881</v>
+        <v>0.04974999904632568</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942062.4699049</v>
+        <v>611942043.6324089</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>181.3001</v>
+        <v>183.9</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>110945157120</v>
+        <v>112536141824</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.48</v>
+        <v>14.69</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.4</v>
+        <v>8.68</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.49</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="6">
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>100933197824</v>
+        <v>100261421056</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>14.169642</v>
+        <v>14.083194</v>
       </c>
       <c r="E6" s="34" t="n">
         <v>10.316</v>
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>365896040448</v>
+        <v>362269278208</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>39.815197</v>
+        <v>39.38654</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>35.294</v>
+        <v>35.488</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>11.623</v>
+        <v>11.687</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>206216478720</v>
+        <v>206943928320</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>41.8125</v>
+        <v>41.96</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>22.34</v>
+        <v>23.296</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.287</v>
+        <v>7.599</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>44411535360</v>
+        <v>44836814848</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.537037</v>
+        <v>13.666666</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.236</v>
+        <v>19.525</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.247</v>
+        <v>4.311</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>237268910080</v>
+        <v>236014616576</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>49.48229</v>
+        <v>49.220707</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>38.44</v>
+        <v>39.186</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>17.139</v>
+        <v>17.472</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>16055473152</v>
+        <v>16170926080</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>11.945846</v>
+        <v>12.031746</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.295</v>
+        <v>9.257999999999999</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.256</v>
+        <v>1.251</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>268130926592</v>
+        <v>270471692288</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>286.0826</v>
+        <v>826.625</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>148.294</v>
+        <v>173.056</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>24.04</v>
+        <v>23.516</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>197847531520</v>
+        <v>194354970624</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>21.146118</v>
+        <v>20.796572</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>16.062</v>
+        <v>16.508</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.373</v>
+        <v>4.495</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-09-19T17:40:52Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-13 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-19 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.866</v>
+        <v>0.867</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>322.14</v>
+        <v>321.07</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>183.9</v>
+        <v>181.29</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.752</v>
+        <v>0.771</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.775</v>
+        <v>0.78</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04974999904632568</v>
+        <v>0.04998000144958496</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942043.6324089</v>
+        <v>611942038.5018479</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>183.9</v>
+        <v>181.29</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>112536141824</v>
+        <v>110938972160</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.69</v>
+        <v>14.47</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.68</v>
+        <v>8.56</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.54</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>100261421056</v>
+        <v>98945695744</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>14.083194</v>
+        <v>13.890625</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>10.316</v>
+        <v>10.194</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.983</v>
+        <v>3.829</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>362269278208</v>
+        <v>352809615360</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>39.38654</v>
+        <v>38.325</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>35.488</v>
+        <v>34.557</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>11.687</v>
+        <v>11.38</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>206943928320</v>
+        <v>191235735552</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>41.96</v>
+        <v>39.166668</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>23.296</v>
+        <v>21.636</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.599</v>
+        <v>7.058</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>44836814848</v>
+        <v>43824717824</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.666666</v>
+        <v>13.358025</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.525</v>
+        <v>19.074</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.311</v>
+        <v>4.211</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>236014616576</v>
+        <v>231245725696</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>49.220707</v>
+        <v>48.357925</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>39.186</v>
+        <v>38.399</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>17.472</v>
+        <v>17.121</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>16170926080</v>
+        <v>16024099840</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>12.031746</v>
+        <v>11.9225025</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.257999999999999</v>
+        <v>9.196999999999999</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.251</v>
+        <v>1.242</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>270471692288</v>
+        <v>297408430080</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>826.625</v>
+        <v>908.9499499999999</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>173.056</v>
+        <v>190.323</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>23.516</v>
+        <v>25.863</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>194354970624</v>
+        <v>189815717888</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>20.796572</v>
+        <v>20.334097</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>16.508</v>
+        <v>16.136</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.495</v>
+        <v>4.393</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-09-20T17:41:06Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-19 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-20 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
         <v>191235735552</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>39.166668</v>
+        <v>38.775</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>21.636</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-10-03T17:40:05Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-20 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-03 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.867</v>
+        <v>0.855</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>321.07</v>
+        <v>304.82</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>181.29</v>
+        <v>198.9</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.771</v>
+        <v>0.533</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04998000144958496</v>
+        <v>0.05276999950408936</v>
       </c>
     </row>
     <row r="6">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>8388769792</v>
+        <v>13396989952</v>
       </c>
     </row>
     <row r="33">
@@ -1199,7 +1199,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>10171567104</v>
+        <v>12837769216</v>
       </c>
     </row>
     <row r="34">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942038.5018479</v>
+        <v>611942070.5077928</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>181.29</v>
+        <v>198.9</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>110938972160</v>
+        <v>121715277824</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.47</v>
+        <v>15.9</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.56</v>
+        <v>8.59</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.51</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>98945695744</v>
+        <v>94481776640</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>13.890625</v>
+        <v>13.263951</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>10.194</v>
+        <v>9.444000000000001</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.829</v>
+        <v>3.606</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>352809615360</v>
+        <v>428574343168</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>38.325</v>
+        <v>46.51507</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>34.557</v>
+        <v>42.017</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>11.38</v>
+        <v>13.837</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>191235735552</v>
+        <v>214440476672</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>38.775</v>
+        <v>43.48</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>21.636</v>
+        <v>24.088</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.058</v>
+        <v>7.858</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>43824717824</v>
+        <v>44715794432</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.358025</v>
+        <v>13.629629</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.074</v>
+        <v>19.471</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.211</v>
+        <v>4.299</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>231245725696</v>
+        <v>269992787968</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>48.357925</v>
+        <v>56.52732</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>38.399</v>
+        <v>44.851</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>17.121</v>
+        <v>19.998</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>16024099840</v>
+        <v>14775452672</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>11.9225025</v>
+        <v>10.9934635</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.196999999999999</v>
+        <v>8.672000000000001</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.242</v>
+        <v>1.171</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>297408430080</v>
+        <v>329850322944</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>908.9499499999999</v>
+        <v>1008.1</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>190.323</v>
+        <v>211.119</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>25.863</v>
+        <v>28.689</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>189815717888</v>
+        <v>197452333056</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>20.334097</v>
+        <v>21.152174</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>16.136</v>
+        <v>16.762</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.393</v>
+        <v>4.564</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-05T17:40:24Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-04 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-05 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.855</v>
+        <v>0.86</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>304.82</v>
+        <v>300.54</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>198.9</v>
+        <v>194.24</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.533</v>
+        <v>0.547</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.72</v>
+        <v>0.746</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.05276999950408936</v>
+        <v>0.05341000080108643</v>
       </c>
     </row>
     <row r="6">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>1.092</v>
+        <v>1.102</v>
       </c>
     </row>
     <row r="8">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942070.5077928</v>
+        <v>611942104.7775947</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>198.9</v>
+        <v>194.24</v>
       </c>
     </row>
     <row r="38">
@@ -1520,10 +1520,10 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>121715277824</v>
+        <v>118863634432</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>15.9</v>
+        <v>15.51</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>8.59</v>
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>94481776640</v>
+        <v>91676016640</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>13.263951</v>
+        <v>13.151865</v>
       </c>
       <c r="E6" s="34" t="n">
         <v>9.444000000000001</v>
@@ -1568,10 +1568,10 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>428574343168</v>
+        <v>425554706432</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>46.51507</v>
+        <v>46.26704</v>
       </c>
       <c r="E7" s="34" t="n">
         <v>42.017</v>
@@ -1592,10 +1592,10 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>214440476672</v>
+        <v>214933684224</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>43.48</v>
+        <v>43.58</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>24.088</v>
@@ -1616,10 +1616,10 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>44715794432</v>
+        <v>43298172928</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.629629</v>
+        <v>13.197531</v>
       </c>
       <c r="E9" s="34" t="n">
         <v>19.471</v>
@@ -1640,10 +1640,10 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>269992787968</v>
+        <v>266749837312</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>56.52732</v>
+        <v>55.84836</v>
       </c>
       <c r="E10" s="34" t="n">
         <v>44.851</v>
@@ -1664,10 +1664,10 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>14775452672</v>
+        <v>14860474368</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>10.9934635</v>
+        <v>11.056723</v>
       </c>
       <c r="E11" s="34" t="n">
         <v>8.672000000000001</v>
@@ -1688,10 +1688,10 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>329850322944</v>
+        <v>332026183680</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>1008.1</v>
+        <v>1014.75</v>
       </c>
       <c r="E12" s="34" t="n">
         <v>211.119</v>
@@ -1712,10 +1712,10 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>197452333056</v>
+        <v>194285535232</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>21.152174</v>
+        <v>21.053818</v>
       </c>
       <c r="E13" s="34" t="n">
         <v>16.762</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-10-06T17:41:48Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-05 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-06 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.86</v>
+        <v>0.863</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>300.54</v>
+        <v>303.23</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>194.24</v>
+        <v>194.33</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.547</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.746</v>
+        <v>0.759</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.05341000080108643</v>
+        <v>0.05276999950408936</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942104.7775947</v>
+        <v>611942104.9143209</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>194.24</v>
+        <v>194.33</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>118863634432</v>
+        <v>118918709248</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>15.51</v>
+        <v>14.33</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.59</v>
+        <v>8.42</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.63</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>91676016640</v>
+        <v>92510896128</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>13.151865</v>
+        <v>13.271636</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>9.444000000000001</v>
+        <v>9.487</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.606</v>
+        <v>3.623</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>425554706432</v>
+        <v>423340605440</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>46.26704</v>
+        <v>46.026318</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>42.017</v>
+        <v>42.193</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>13.837</v>
+        <v>13.895</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>214933684224</v>
+        <v>221197221888</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>43.58</v>
+        <v>44.85</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>24.088</v>
+        <v>24.169</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.858</v>
+        <v>7.884</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>43298172928</v>
+        <v>42629865472</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.197531</v>
+        <v>12.993827</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.471</v>
+        <v>18.965</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.299</v>
+        <v>4.188</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>266749837312</v>
+        <v>259787653120</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>55.84836</v>
+        <v>54.390713</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>44.851</v>
+        <v>44.842</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>19.998</v>
+        <v>19.994</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>14860474368</v>
+        <v>14765413376</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>11.056723</v>
+        <v>10.985994</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.672000000000001</v>
+        <v>8.762</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.171</v>
+        <v>1.184</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>332026183680</v>
+        <v>341351399424</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>1014.75</v>
+        <v>1043.25</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>211.119</v>
+        <v>212.965</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>28.689</v>
+        <v>28.94</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>194285535232</v>
+        <v>194069151744</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>21.053818</v>
+        <v>21.034721</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>16.762</v>
+        <v>16.405</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.564</v>
+        <v>4.467</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-07T17:42:08Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-06 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-07 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.863</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>303.23</v>
+        <v>303.31</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>194.33</v>
+        <v>197.085</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.539</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.759</v>
+        <v>0.753</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.778</v>
+        <v>0.333</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.05276999950408936</v>
+        <v>0.05275000095367432</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942104.9143209</v>
+        <v>611942088.2563361</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>194.33</v>
+        <v>197.085</v>
       </c>
     </row>
     <row r="38">
@@ -1520,208 +1520,208 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>118918709248</v>
+        <v>120604606464</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.33</v>
+        <v>14.53</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.42</v>
+        <v>8.35</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.6</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>CACI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Adobe Inc.</t>
+          <t>CACI International, Inc.</t>
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>92510896128</v>
+        <v>13022407680</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>13.271636</v>
+        <v>24.389902</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>9.487</v>
+        <v>15.511</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.623</v>
+        <v>1.928</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>CGEMY</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Applied Materials, Inc.</t>
+          <t>Capgemini SE</t>
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>423340605440</v>
+        <v>20534472704</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>46.026318</v>
+        <v>13.445652</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>42.193</v>
+        <v>9.297000000000001</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>13.895</v>
+        <v>1.223</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>CTSH</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Amphenol Corporation</t>
+          <t xml:space="preserve">Cognizant Technology Solutions </t>
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>221197221888</v>
+        <v>25711357952</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>44.85</v>
+        <v>12.275269</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>24.169</v>
+        <v>6.645</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.884</v>
+        <v>1.239</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>DXC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Infosys Limited</t>
+          <t>DXC Technology Company</t>
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>42629865472</v>
+        <v>1889382912</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>12.993827</v>
+        <v>15.559211</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>18.965</v>
+        <v>3.203</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.188</v>
+        <v>0.351</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>EPAM</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KLA Corporation</t>
+          <t>EPAM Systems, Inc.</t>
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>259787653120</v>
+        <v>5606730752</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>54.390713</v>
+        <v>14.746947</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>44.842</v>
+        <v>6.64</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>19.994</v>
+        <v>0.891</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LDOS</t>
+          <t>GIB</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Leidos Holdings, Inc.</t>
+          <t>CGI Inc.</t>
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>14765413376</v>
+        <v>14519092224</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>10.985994</v>
+        <v>12.04725</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.762</v>
+        <v>6.19</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.184</v>
+        <v>1.099</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>GLOB</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Palo Alto Networks, Inc.</t>
+          <t>Globant S.A.</t>
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>341351399424</v>
+        <v>1538487680</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>1043.25</v>
+        <v>13.91797</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>212.965</v>
+        <v>4.943</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>28.94</v>
+        <v>0.789</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>QUALCOMM Incorporated</t>
+          <t>International Business Machines</t>
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>194069151744</v>
+        <v>207542779904</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>21.034721</v>
+        <v>19.581333</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>16.405</v>
+        <v>16.13</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.467</v>
+        <v>3.846</v>
       </c>
     </row>
     <row r="15">
@@ -1772,10 +1772,10 @@
         <v>0.5</v>
       </c>
       <c r="E17" s="36" t="n">
-        <v>0</v>
+        <v>0.667</v>
       </c>
       <c r="F17" s="36" t="n">
-        <v>0.167</v>
+        <v>0.833</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-26T17:42:05Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-07 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-26 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.577</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>303.31</v>
+        <v>350.44</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>197.085</v>
+        <v>244.8</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.539</v>
+        <v>0.432</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.753</v>
+        <v>0.577</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.333</v>
+        <v>0.222</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>1</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.05275000095367432</v>
+        <v>0.0498199987411499</v>
       </c>
     </row>
     <row r="6">
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>0.05241951788891955</v>
+        <v>0.06058952448549225</v>
       </c>
     </row>
     <row r="12">
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>10874360000</v>
+        <v>11620598000</v>
       </c>
     </row>
     <row r="15">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942088.2563361</v>
+        <v>611942065.359477</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>197.085</v>
+        <v>244.8</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>120604606464</v>
+        <v>149803417600</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.53</v>
+        <v>18.05</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.35</v>
+        <v>11.14</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.58</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>13022407680</v>
+        <v>14793800704</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>24.389902</v>
+        <v>27.48009</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>15.511</v>
+        <v>15.276</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.928</v>
+        <v>1.956</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>20534472704</v>
+        <v>23016204288</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>13.445652</v>
+        <v>15.070652</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>9.297000000000001</v>
+        <v>10.149</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>1.223</v>
+        <v>1.335</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>25711357952</v>
+        <v>30846420992</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>12.275269</v>
+        <v>14.726882</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>6.645</v>
+        <v>8.131</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>1.239</v>
+        <v>1.516</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>1889382912</v>
+        <v>2581224704</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>15.559211</v>
+        <v>21.25658</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>3.203</v>
+        <v>3.701</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.351</v>
+        <v>0.405</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>5606730752</v>
+        <v>7007059456</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>14.746947</v>
+        <v>18.430122</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>6.64</v>
+        <v>8.484999999999999</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>0.891</v>
+        <v>1.138</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>14519092224</v>
+        <v>16878737408</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>12.04725</v>
+        <v>14.005172</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>6.19</v>
+        <v>7.058</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.099</v>
+        <v>1.253</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>1538487680</v>
+        <v>1917604096</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>13.91797</v>
+        <v>17.347656</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>4.943</v>
+        <v>5.981</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>0.789</v>
+        <v>0.954</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>207542779904</v>
+        <v>238756413440</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>19.581333</v>
+        <v>21.554607</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>16.13</v>
+        <v>17.819</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>3.846</v>
+        <v>4.242</v>
       </c>
     </row>
     <row r="15">
@@ -1772,10 +1772,10 @@
         <v>0.5</v>
       </c>
       <c r="E17" s="36" t="n">
-        <v>0.667</v>
+        <v>0.833</v>
       </c>
       <c r="F17" s="36" t="n">
-        <v>0.833</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">

</xml_diff>